<commit_message>
feat: implementar pipeline de observacao Lay Under 1.5 FT, dashboard Streamlit e regras GEMINI.md atualizadas
</commit_message>
<xml_diff>
--- a/sinais_gerados/sinais_gerados_2026-08-23.xlsx
+++ b/sinais_gerados/sinais_gerados_2026-08-23.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,30 +566,30 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>PORTUGAL 1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Valladolid</t>
+          <t>Famalicao</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>25.64</v>
+        <v>28.57</v>
       </c>
       <c r="H4" t="n">
         <v>200</v>
       </c>
       <c r="I4" t="n">
-        <v>24.36</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="5">
@@ -605,30 +605,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="G5" t="n">
-        <v>28.57</v>
+        <v>14.81</v>
       </c>
       <c r="H5" t="n">
         <v>200</v>
       </c>
       <c r="I5" t="n">
-        <v>27.14</v>
+        <v>14.07</v>
       </c>
     </row>
     <row r="6">
@@ -756,35 +756,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 0x0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>West Brom</t>
+          <t>Racing Club</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11</v>
+        <v>8.4</v>
       </c>
       <c r="G9" t="n">
-        <v>20</v>
+        <v>27.03</v>
       </c>
       <c r="H9" t="n">
         <v>200</v>
       </c>
       <c r="I9" t="n">
-        <v>19</v>
+        <v>25.68</v>
       </c>
     </row>
     <row r="10">
@@ -800,30 +800,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>ENGLAND 2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Chongqing Tonglianglong</t>
+          <t>West Brom</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Dalian Yingbo</t>
+          <t>Burnley</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G10" t="n">
-        <v>18.18</v>
+        <v>20</v>
       </c>
       <c r="H10" t="n">
         <v>200</v>
       </c>
       <c r="I10" t="n">
-        <v>17.27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -839,30 +839,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FRANCE 1</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Chongqing Tonglianglong</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Dalian Yingbo</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>7.8</v>
+        <v>12</v>
       </c>
       <c r="G11" t="n">
-        <v>29.41</v>
+        <v>18.18</v>
       </c>
       <c r="H11" t="n">
         <v>200</v>
       </c>
       <c r="I11" t="n">
-        <v>27.94</v>
+        <v>17.27</v>
       </c>
     </row>
     <row r="12">
@@ -878,30 +878,30 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>FRANCE 1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bandirmaspor</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Keciorengucu</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>11.5</v>
+        <v>7.8</v>
       </c>
       <c r="G12" t="n">
-        <v>19.05</v>
+        <v>29.41</v>
       </c>
       <c r="H12" t="n">
         <v>200</v>
       </c>
       <c r="I12" t="n">
-        <v>18.1</v>
+        <v>27.94</v>
       </c>
     </row>
     <row r="13">
@@ -917,30 +917,30 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Bandirmaspor</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Valladolid</t>
+          <t>Keciorengucu</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>12.5</v>
+        <v>11.5</v>
       </c>
       <c r="G13" t="n">
-        <v>17.39</v>
+        <v>19.05</v>
       </c>
       <c r="H13" t="n">
         <v>200</v>
       </c>
       <c r="I13" t="n">
-        <v>16.52</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="14">
@@ -956,30 +956,30 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>SPAIN 2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Valladolid</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="G14" t="n">
-        <v>22.73</v>
+        <v>17.39</v>
       </c>
       <c r="H14" t="n">
         <v>200</v>
       </c>
       <c r="I14" t="n">
-        <v>21.59</v>
+        <v>16.52</v>
       </c>
     </row>
     <row r="15">
@@ -1000,25 +1000,25 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>15.38</v>
+        <v>22.73</v>
       </c>
       <c r="H15" t="n">
         <v>200</v>
       </c>
       <c r="I15" t="n">
-        <v>14.61</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="16">
@@ -1034,30 +1034,30 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G16" t="n">
-        <v>28.57</v>
+        <v>15.38</v>
       </c>
       <c r="H16" t="n">
         <v>200</v>
       </c>
       <c r="I16" t="n">
-        <v>27.14</v>
+        <v>14.61</v>
       </c>
     </row>
     <row r="17">
@@ -1073,30 +1073,30 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ISRAEL 1</t>
+          <t>PORTUGAL 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hapoel Jerusalem</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Maccabi Tel Aviv</t>
+          <t>Famalicao</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G17" t="n">
-        <v>25</v>
+        <v>28.57</v>
       </c>
       <c r="H17" t="n">
         <v>200</v>
       </c>
       <c r="I17" t="n">
-        <v>23.75</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="18">
@@ -1112,30 +1112,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ISRAEL 1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Hapoel Jerusalem</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Maccabi Tel Aviv</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.5</v>
+        <v>9</v>
       </c>
       <c r="G18" t="n">
-        <v>19.05</v>
+        <v>25</v>
       </c>
       <c r="H18" t="n">
         <v>200</v>
       </c>
       <c r="I18" t="n">
-        <v>18.1</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="19">
@@ -1151,30 +1151,30 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ROMANIA 1</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="G19" t="n">
-        <v>21.05</v>
+        <v>19.05</v>
       </c>
       <c r="H19" t="n">
         <v>200</v>
       </c>
       <c r="I19" t="n">
-        <v>20</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="20">
@@ -1190,30 +1190,30 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>ROMANIA 1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>8.6</v>
+        <v>10.5</v>
       </c>
       <c r="G20" t="n">
-        <v>26.32</v>
+        <v>21.05</v>
       </c>
       <c r="H20" t="n">
         <v>200</v>
       </c>
       <c r="I20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -1229,30 +1229,30 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="G21" t="n">
-        <v>31.25</v>
+        <v>26.32</v>
       </c>
       <c r="H21" t="n">
         <v>200</v>
       </c>
       <c r="I21" t="n">
-        <v>29.69</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22">
@@ -1268,30 +1268,30 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="G22" t="n">
-        <v>32.26</v>
+        <v>31.25</v>
       </c>
       <c r="H22" t="n">
         <v>200</v>
       </c>
       <c r="I22" t="n">
-        <v>30.65</v>
+        <v>29.69</v>
       </c>
     </row>
     <row r="23">
@@ -1307,30 +1307,30 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Grosseto</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Spezia</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
       <c r="G23" t="n">
-        <v>23.26</v>
+        <v>32.26</v>
       </c>
       <c r="H23" t="n">
         <v>200</v>
       </c>
       <c r="I23" t="n">
-        <v>22.1</v>
+        <v>30.65</v>
       </c>
     </row>
     <row r="24">
@@ -1351,25 +1351,25 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sambenedettese</t>
+          <t>Grosseto</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Forli</t>
+          <t>Spezia</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="G24" t="n">
-        <v>22.73</v>
+        <v>23.26</v>
       </c>
       <c r="H24" t="n">
         <v>200</v>
       </c>
       <c r="I24" t="n">
-        <v>21.59</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="25">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Sambenedettese</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Forli</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1424,30 +1424,30 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>SPAIN 2</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Delfin</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>28.57</v>
+        <v>22.73</v>
       </c>
       <c r="H26" t="n">
         <v>200</v>
       </c>
       <c r="I26" t="n">
-        <v>27.14</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="27">
@@ -1463,30 +1463,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Belgrano</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Defensa y Justicia</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>7.6</v>
+        <v>14.5</v>
       </c>
       <c r="G27" t="n">
-        <v>30.3</v>
+        <v>14.81</v>
       </c>
       <c r="H27" t="n">
         <v>200</v>
       </c>
       <c r="I27" t="n">
-        <v>28.79</v>
+        <v>14.07</v>
       </c>
     </row>
     <row r="28">
@@ -1502,30 +1502,30 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Delfin</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Envigado</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>9.6</v>
+        <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>23.26</v>
+        <v>28.57</v>
       </c>
       <c r="H28" t="n">
         <v>200</v>
       </c>
       <c r="I28" t="n">
-        <v>22.1</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="29">
@@ -1541,30 +1541,30 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>BRAZIL 1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Racing Club</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="G29" t="n">
-        <v>29.41</v>
+        <v>30.3</v>
       </c>
       <c r="H29" t="n">
         <v>200</v>
       </c>
       <c r="I29" t="n">
-        <v>27.94</v>
+        <v>28.79</v>
       </c>
     </row>
     <row r="30">
@@ -1575,22 +1575,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEXICO 1</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Cruz Azul</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Envigado</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1614,35 +1614,35 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SWEDEN 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Racing Club</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Degerfors</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>7.8</v>
       </c>
       <c r="G31" t="n">
-        <v>22.22</v>
+        <v>29.41</v>
       </c>
       <c r="H31" t="n">
         <v>200</v>
       </c>
       <c r="I31" t="n">
-        <v>21.11</v>
+        <v>27.94</v>
       </c>
     </row>
     <row r="32">
@@ -1658,30 +1658,30 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BOSNIA 1</t>
+          <t>MEXICO 1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Borac Banja Luka</t>
+          <t>Cruz Azul</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Celik Zenica</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>8</v>
+        <v>9.6</v>
       </c>
       <c r="G32" t="n">
-        <v>28.57</v>
+        <v>23.26</v>
       </c>
       <c r="H32" t="n">
         <v>200</v>
       </c>
       <c r="I32" t="n">
-        <v>27.14</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="33">
@@ -1697,30 +1697,30 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>SPAIN 2</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Valladolid</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G33" t="n">
-        <v>28.57</v>
+        <v>33.33</v>
       </c>
       <c r="H33" t="n">
         <v>200</v>
       </c>
       <c r="I33" t="n">
-        <v>27.14</v>
+        <v>31.66</v>
       </c>
     </row>
     <row r="34">
@@ -1736,30 +1736,30 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ITALY 2</t>
+          <t>BOSNIA 1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Pisa</t>
+          <t>Borac Banja Luka</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Padova</t>
+          <t>Celik Zenica</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="G34" t="n">
-        <v>29.41</v>
+        <v>28.57</v>
       </c>
       <c r="H34" t="n">
         <v>200</v>
       </c>
       <c r="I34" t="n">
-        <v>27.94</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="35">
@@ -1775,30 +1775,30 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ITALY 2</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Verona</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Ascoli</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="G35" t="n">
-        <v>27.03</v>
+        <v>28.57</v>
       </c>
       <c r="H35" t="n">
         <v>200</v>
       </c>
       <c r="I35" t="n">
-        <v>25.68</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="36">
@@ -1814,30 +1814,30 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Pisa</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="G36" t="n">
-        <v>27.78</v>
+        <v>29.41</v>
       </c>
       <c r="H36" t="n">
         <v>200</v>
       </c>
       <c r="I36" t="n">
-        <v>26.39</v>
+        <v>27.94</v>
       </c>
     </row>
     <row r="37">
@@ -1853,17 +1853,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Verona</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Ascoli</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1892,30 +1892,30 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>PORTUGAL 1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Goztepe</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Genclerbirligi</t>
+          <t>Famalicao</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G38" t="n">
-        <v>27.03</v>
+        <v>27.78</v>
       </c>
       <c r="H38" t="n">
         <v>200</v>
       </c>
       <c r="I38" t="n">
-        <v>25.68</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="39">
@@ -1931,30 +1931,30 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ITALY 2</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Juve Stabia</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>7.6</v>
+        <v>8.4</v>
       </c>
       <c r="G39" t="n">
-        <v>30.3</v>
+        <v>27.03</v>
       </c>
       <c r="H39" t="n">
         <v>200</v>
       </c>
       <c r="I39" t="n">
-        <v>28.79</v>
+        <v>25.68</v>
       </c>
     </row>
     <row r="40">
@@ -1970,30 +1970,30 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sambenedettese</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Forli</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="G40" t="n">
-        <v>28.57</v>
+        <v>27.03</v>
       </c>
       <c r="H40" t="n">
         <v>200</v>
       </c>
       <c r="I40" t="n">
-        <v>27.14</v>
+        <v>25.68</v>
       </c>
     </row>
     <row r="41">
@@ -2009,30 +2009,30 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Belgrano</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Defensa y Justicia</t>
+          <t>Juve Stabia</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>7</v>
+        <v>7.6</v>
       </c>
       <c r="G41" t="n">
-        <v>33.33</v>
+        <v>30.3</v>
       </c>
       <c r="H41" t="n">
         <v>200</v>
       </c>
       <c r="I41" t="n">
-        <v>31.66</v>
+        <v>28.79</v>
       </c>
     </row>
     <row r="42">
@@ -2048,30 +2048,30 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Delfin</t>
+          <t>Sambenedettese</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Forli</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>9.6</v>
+        <v>8</v>
       </c>
       <c r="G42" t="n">
-        <v>23.26</v>
+        <v>28.57</v>
       </c>
       <c r="H42" t="n">
         <v>200</v>
       </c>
       <c r="I42" t="n">
-        <v>22.1</v>
+        <v>27.14</v>
       </c>
     </row>
     <row r="43">
@@ -2087,30 +2087,30 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BRAZIL 3</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Maranhao</t>
+          <t>Belgrano</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Itabaiana</t>
+          <t>Defensa y Justicia</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="G43" t="n">
-        <v>34.48</v>
+        <v>33.33</v>
       </c>
       <c r="H43" t="n">
         <v>200</v>
       </c>
       <c r="I43" t="n">
-        <v>32.76</v>
+        <v>31.66</v>
       </c>
     </row>
     <row r="44">
@@ -2126,30 +2126,30 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>URUGUAY 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Nacional (Uru)</t>
+          <t>Delfin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="G44" t="n">
-        <v>29.41</v>
+        <v>23.26</v>
       </c>
       <c r="H44" t="n">
         <v>200</v>
       </c>
       <c r="I44" t="n">
-        <v>27.94</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="45">
@@ -2165,30 +2165,30 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>BRAZIL 3</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Maranhao</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Itabaiana</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>8.4</v>
+        <v>6.8</v>
       </c>
       <c r="G45" t="n">
-        <v>27.03</v>
+        <v>34.48</v>
       </c>
       <c r="H45" t="n">
         <v>200</v>
       </c>
       <c r="I45" t="n">
-        <v>25.68</v>
+        <v>32.76</v>
       </c>
     </row>
     <row r="46">
@@ -2204,30 +2204,30 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>URUGUAY 1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nacional (Uru)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Envigado</t>
+          <t>Progreso</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>7.2</v>
+        <v>7.8</v>
       </c>
       <c r="G46" t="n">
-        <v>32.26</v>
+        <v>29.41</v>
       </c>
       <c r="H46" t="n">
         <v>200</v>
       </c>
       <c r="I46" t="n">
-        <v>30.65</v>
+        <v>27.94</v>
       </c>
     </row>
     <row r="47">
@@ -2238,35 +2238,35 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MEXICO 1</t>
+          <t>BRAZIL 1</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Cruz Azul</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.800000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="G47" t="n">
-        <v>22.73</v>
+        <v>27.03</v>
       </c>
       <c r="H47" t="n">
         <v>200</v>
       </c>
       <c r="I47" t="n">
-        <v>21.59</v>
+        <v>25.68</v>
       </c>
     </row>
     <row r="48">
@@ -2277,35 +2277,35 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Chongqing Tonglianglong</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Dalian Yingbo</t>
+          <t>Envigado</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>14</v>
+        <v>7.2</v>
       </c>
       <c r="G48" t="n">
-        <v>15.38</v>
+        <v>32.26</v>
       </c>
       <c r="H48" t="n">
         <v>200</v>
       </c>
       <c r="I48" t="n">
-        <v>14.61</v>
+        <v>30.65</v>
       </c>
     </row>
     <row r="49">
@@ -2321,30 +2321,30 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ENGLAND 1</t>
+          <t>MEXICO 1</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Cruz Azul</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>12.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G49" t="n">
-        <v>17.39</v>
+        <v>22.73</v>
       </c>
       <c r="H49" t="n">
         <v>200</v>
       </c>
       <c r="I49" t="n">
-        <v>16.52</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="50">
@@ -2360,30 +2360,30 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SWEDEN 1</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Chongqing Tonglianglong</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Degerfors</t>
+          <t>Dalian Yingbo</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G50" t="n">
-        <v>16.67</v>
+        <v>15.38</v>
       </c>
       <c r="H50" t="n">
         <v>200</v>
       </c>
       <c r="I50" t="n">
-        <v>15.84</v>
+        <v>14.61</v>
       </c>
     </row>
     <row r="51">
@@ -2399,30 +2399,30 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CHILE 1</t>
+          <t>ENGLAND 1</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>La Serena</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Cobresal</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="G51" t="n">
-        <v>18.18</v>
+        <v>17.39</v>
       </c>
       <c r="H51" t="n">
         <v>200</v>
       </c>
       <c r="I51" t="n">
-        <v>17.27</v>
+        <v>16.52</v>
       </c>
     </row>
     <row r="52">
@@ -2438,30 +2438,30 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>POLAND 2</t>
+          <t>SWEDEN 1</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Brommapojkarna</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Degerfors</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="G52" t="n">
-        <v>16</v>
+        <v>16.67</v>
       </c>
       <c r="H52" t="n">
         <v>200</v>
       </c>
       <c r="I52" t="n">
-        <v>15.2</v>
+        <v>15.84</v>
       </c>
     </row>
     <row r="53">
@@ -2477,30 +2477,30 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>POLAND 1</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G53" t="n">
-        <v>25</v>
+        <v>14.29</v>
       </c>
       <c r="H53" t="n">
         <v>200</v>
       </c>
       <c r="I53" t="n">
-        <v>23.75</v>
+        <v>13.58</v>
       </c>
     </row>
     <row r="54">
@@ -2516,30 +2516,30 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BOSNIA 1</t>
+          <t>CHILE 1</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Zrinjski</t>
+          <t>La Serena</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Zeljeznicar</t>
+          <t>Cobresal</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>6.8</v>
+        <v>12</v>
       </c>
       <c r="G54" t="n">
-        <v>34.48</v>
+        <v>18.18</v>
       </c>
       <c r="H54" t="n">
         <v>200</v>
       </c>
       <c r="I54" t="n">
-        <v>32.76</v>
+        <v>17.27</v>
       </c>
     </row>
     <row r="55">
@@ -2555,30 +2555,30 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ITALY 2</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Juve Stabia</t>
+          <t>Basaksehir</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>8.199999999999999</v>
+        <v>15</v>
       </c>
       <c r="G55" t="n">
-        <v>27.78</v>
+        <v>14.29</v>
       </c>
       <c r="H55" t="n">
         <v>200</v>
       </c>
       <c r="I55" t="n">
-        <v>26.39</v>
+        <v>13.58</v>
       </c>
     </row>
     <row r="56">
@@ -2594,30 +2594,30 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ICELAND 1</t>
+          <t>POLAND 2</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Vikingur Reykjavik</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Valur</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="F56" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G56" t="n">
         <v>16</v>
       </c>
-      <c r="G56" t="n">
-        <v>13.33</v>
-      </c>
       <c r="H56" t="n">
         <v>200</v>
       </c>
       <c r="I56" t="n">
-        <v>12.66</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="57">
@@ -2633,30 +2633,30 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Belgrano</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Defensa y Justicia</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="G57" t="n">
-        <v>21.05</v>
+        <v>20</v>
       </c>
       <c r="H57" t="n">
         <v>200</v>
       </c>
       <c r="I57" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58">
@@ -2672,30 +2672,30 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G58" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H58" t="n">
         <v>200</v>
       </c>
       <c r="I58" t="n">
-        <v>19</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="59">
@@ -2711,30 +2711,30 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>BOSNIA 1</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>River Plate</t>
+          <t>Zrinjski</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Velez Sarsfield</t>
+          <t>Zeljeznicar</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>8.800000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G59" t="n">
-        <v>25.64</v>
+        <v>34.48</v>
       </c>
       <c r="H59" t="n">
         <v>200</v>
       </c>
       <c r="I59" t="n">
-        <v>24.36</v>
+        <v>32.76</v>
       </c>
     </row>
     <row r="60">
@@ -2745,35 +2745,35 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FRANCE 1</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Juve Stabia</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>9.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G60" t="n">
-        <v>23.26</v>
+        <v>27.78</v>
       </c>
       <c r="H60" t="n">
         <v>200</v>
       </c>
       <c r="I60" t="n">
-        <v>22.1</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="61">
@@ -2784,35 +2784,35 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FRANCE 1</t>
+          <t>ICELAND 1</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Vikingur Reykjavik</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Valur</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>13.5</v>
+        <v>16</v>
       </c>
       <c r="G61" t="n">
-        <v>16</v>
+        <v>13.33</v>
       </c>
       <c r="H61" t="n">
         <v>200</v>
       </c>
       <c r="I61" t="n">
-        <v>15.2</v>
+        <v>12.66</v>
       </c>
     </row>
     <row r="62">
@@ -2823,35 +2823,35 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ENGLAND 1</t>
+          <t>BRAZIL 1</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Newcastle</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>14.5</v>
+        <v>11</v>
       </c>
       <c r="G62" t="n">
-        <v>14.81</v>
+        <v>20</v>
       </c>
       <c r="H62" t="n">
         <v>200</v>
       </c>
       <c r="I62" t="n">
-        <v>14.07</v>
+        <v>19</v>
       </c>
     </row>
     <row r="63">
@@ -2862,35 +2862,35 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>River Plate</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Velez Sarsfield</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G63" t="n">
-        <v>25</v>
+        <v>25.64</v>
       </c>
       <c r="H63" t="n">
         <v>200</v>
       </c>
       <c r="I63" t="n">
-        <v>23.75</v>
+        <v>24.36</v>
       </c>
     </row>
     <row r="64">
@@ -2906,30 +2906,30 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ISRAEL 1</t>
+          <t>FRANCE 1</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Hapoel Jerusalem</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Maccabi Tel Aviv</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="G64" t="n">
-        <v>22.73</v>
+        <v>23.26</v>
       </c>
       <c r="H64" t="n">
         <v>200</v>
       </c>
       <c r="I64" t="n">
-        <v>21.59</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="65">
@@ -2945,17 +2945,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ROMANIA 1</t>
+          <t>FRANCE 1</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -2984,30 +2984,30 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>ENGLAND 1</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>Newcastle</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>10.5</v>
+        <v>14.5</v>
       </c>
       <c r="G66" t="n">
-        <v>21.05</v>
+        <v>14.81</v>
       </c>
       <c r="H66" t="n">
         <v>200</v>
       </c>
       <c r="I66" t="n">
-        <v>20</v>
+        <v>14.07</v>
       </c>
     </row>
     <row r="67">
@@ -3028,25 +3028,25 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="G67" t="n">
-        <v>22.73</v>
+        <v>25</v>
       </c>
       <c r="H67" t="n">
         <v>200</v>
       </c>
       <c r="I67" t="n">
-        <v>21.59</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="68">
@@ -3062,30 +3062,30 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ISRAEL 1</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Hapoel Jerusalem</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Maccabi Tel Aviv</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>12</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G68" t="n">
-        <v>18.18</v>
+        <v>22.73</v>
       </c>
       <c r="H68" t="n">
         <v>200</v>
       </c>
       <c r="I68" t="n">
-        <v>17.27</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="69">
@@ -3101,30 +3101,30 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ROMANIA 1</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>9.199999999999999</v>
+        <v>13.5</v>
       </c>
       <c r="G69" t="n">
-        <v>24.39</v>
+        <v>16</v>
       </c>
       <c r="H69" t="n">
         <v>200</v>
       </c>
       <c r="I69" t="n">
-        <v>23.17</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="70">
@@ -3140,30 +3140,30 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Delfin</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>15.5</v>
+        <v>10.5</v>
       </c>
       <c r="G70" t="n">
-        <v>13.79</v>
+        <v>21.05</v>
       </c>
       <c r="H70" t="n">
         <v>200</v>
       </c>
       <c r="I70" t="n">
-        <v>13.1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="71">
@@ -3174,35 +3174,35 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SOUTH KOREA 1</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Gwangju FC</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Incheon Utd</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G71" t="n">
-        <v>10</v>
+        <v>22.73</v>
       </c>
       <c r="H71" t="n">
         <v>200</v>
       </c>
       <c r="I71" t="n">
-        <v>9.5</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="72">
@@ -3213,35 +3213,35 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SOUTH KOREA 2</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Jeonnam Dragons</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Hwaseong FC</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="G72" t="n">
-        <v>8</v>
+        <v>18.18</v>
       </c>
       <c r="H72" t="n">
         <v>200</v>
       </c>
       <c r="I72" t="n">
-        <v>7.6</v>
+        <v>17.27</v>
       </c>
     </row>
     <row r="73">
@@ -3252,35 +3252,35 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FRANCE 1</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Elche</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>19</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G73" t="n">
-        <v>11.11</v>
+        <v>24.39</v>
       </c>
       <c r="H73" t="n">
         <v>200</v>
       </c>
       <c r="I73" t="n">
-        <v>10.55</v>
+        <v>23.17</v>
       </c>
     </row>
     <row r="74">
@@ -3291,35 +3291,35 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>AC Horsens</t>
+          <t>Delfin</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>29</v>
+        <v>15.5</v>
       </c>
       <c r="G74" t="n">
-        <v>7.14</v>
+        <v>13.79</v>
       </c>
       <c r="H74" t="n">
         <v>200</v>
       </c>
       <c r="I74" t="n">
-        <v>6.78</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="75">
@@ -3335,30 +3335,30 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>FINLAND 1</t>
+          <t>SOUTH KOREA 1</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Gwangju FC</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FC Inter Turku</t>
+          <t>Incheon Utd</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G75" t="n">
-        <v>9.09</v>
+        <v>10</v>
       </c>
       <c r="H75" t="n">
         <v>200</v>
       </c>
       <c r="I75" t="n">
-        <v>8.640000000000001</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="76">
@@ -3374,30 +3374,30 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>SOUTH KOREA 2</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Van Buyuksehir Belediyespor</t>
+          <t>Jeonnam Dragons</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Istanbulspor</t>
+          <t>Hwaseong FC</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G76" t="n">
-        <v>7.41</v>
+        <v>8</v>
       </c>
       <c r="H76" t="n">
         <v>200</v>
       </c>
       <c r="I76" t="n">
-        <v>7.04</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="77">
@@ -3413,30 +3413,30 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>FRANCE 1</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G77" t="n">
-        <v>10</v>
+        <v>11.11</v>
       </c>
       <c r="H77" t="n">
         <v>200</v>
       </c>
       <c r="I77" t="n">
-        <v>9.5</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="78">
@@ -3452,30 +3452,30 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>DENMARK 1</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G78" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H78" t="n">
         <v>200</v>
       </c>
       <c r="I78" t="n">
-        <v>9.5</v>
+        <v>6.78</v>
       </c>
     </row>
     <row r="79">
@@ -3491,17 +3491,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>FINLAND 1</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Grosseto</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Spezia</t>
+          <t>FC Inter Turku</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -3530,30 +3530,30 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Chapecoense</t>
+          <t>Van Buyuksehir Belediyespor</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Sao Paulo</t>
+          <t>Istanbulspor</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G80" t="n">
-        <v>8.33</v>
+        <v>7.41</v>
       </c>
       <c r="H80" t="n">
         <v>200</v>
       </c>
       <c r="I80" t="n">
-        <v>7.91</v>
+        <v>7.04</v>
       </c>
     </row>
     <row r="81">
@@ -3564,35 +3564,35 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ROMANIA 2</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>CSC 1599 Selimbar</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>CS Afumati</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>17.5</v>
+        <v>21</v>
       </c>
       <c r="G81" t="n">
-        <v>12.12</v>
+        <v>10</v>
       </c>
       <c r="H81" t="n">
         <v>200</v>
       </c>
       <c r="I81" t="n">
-        <v>11.51</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="82">
@@ -3603,35 +3603,35 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SOUTH KOREA 1</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Daejeon Citizen</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Gangwon</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>19.5</v>
+        <v>21</v>
       </c>
       <c r="G82" t="n">
-        <v>10.81</v>
+        <v>10</v>
       </c>
       <c r="H82" t="n">
         <v>200</v>
       </c>
       <c r="I82" t="n">
-        <v>10.27</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="83">
@@ -3642,35 +3642,35 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SOUTH KOREA 2</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Chungnam Asan</t>
+          <t>Grosseto</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Yongin FC</t>
+          <t>Spezia</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G83" t="n">
-        <v>11.11</v>
+        <v>9.09</v>
       </c>
       <c r="H83" t="n">
         <v>200</v>
       </c>
       <c r="I83" t="n">
-        <v>10.55</v>
+        <v>8.640000000000001</v>
       </c>
     </row>
     <row r="84">
@@ -3681,35 +3681,35 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>BRAZIL 1</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>West Brom</t>
+          <t>Chapecoense</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Sao Paulo</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>17.5</v>
+        <v>25</v>
       </c>
       <c r="G84" t="n">
-        <v>12.12</v>
+        <v>8.33</v>
       </c>
       <c r="H84" t="n">
         <v>200</v>
       </c>
       <c r="I84" t="n">
-        <v>11.51</v>
+        <v>7.91</v>
       </c>
     </row>
     <row r="85">
@@ -3725,30 +3725,30 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>ROMANIA 2</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Chongqing Tonglianglong</t>
+          <t>CSC 1599 Selimbar</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Dalian Yingbo</t>
+          <t>CS Afumati</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>18.5</v>
+        <v>17.5</v>
       </c>
       <c r="G85" t="n">
-        <v>11.43</v>
+        <v>12.12</v>
       </c>
       <c r="H85" t="n">
         <v>200</v>
       </c>
       <c r="I85" t="n">
-        <v>10.86</v>
+        <v>11.51</v>
       </c>
     </row>
     <row r="86">
@@ -3764,30 +3764,30 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>POLAND 1</t>
+          <t>SOUTH KOREA 1</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Daejeon Citizen</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Gangwon</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>17</v>
+        <v>19.5</v>
       </c>
       <c r="G86" t="n">
-        <v>12.5</v>
+        <v>10.81</v>
       </c>
       <c r="H86" t="n">
         <v>200</v>
       </c>
       <c r="I86" t="n">
-        <v>11.88</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="87">
@@ -3803,30 +3803,30 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ENGLAND 1</t>
+          <t>SOUTH KOREA 2</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Chungnam Asan</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Yongin FC</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G87" t="n">
-        <v>12.5</v>
+        <v>11.11</v>
       </c>
       <c r="H87" t="n">
         <v>200</v>
       </c>
       <c r="I87" t="n">
-        <v>11.88</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="88">
@@ -3842,30 +3842,30 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PORTUGAL 2</t>
+          <t>ENGLAND 2</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Penafiel</t>
+          <t>West Brom</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Sporting Lisbon B</t>
+          <t>Burnley</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="G88" t="n">
-        <v>10.53</v>
+        <v>12.12</v>
       </c>
       <c r="H88" t="n">
         <v>200</v>
       </c>
       <c r="I88" t="n">
-        <v>10</v>
+        <v>11.51</v>
       </c>
     </row>
     <row r="89">
@@ -3881,30 +3881,30 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>VENEZUELA 1</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Monagas</t>
+          <t>Chongqing Tonglianglong</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Portuguesa FC</t>
+          <t>Dalian Yingbo</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="G89" t="n">
-        <v>11.11</v>
+        <v>11.43</v>
       </c>
       <c r="H89" t="n">
         <v>200</v>
       </c>
       <c r="I89" t="n">
-        <v>10.55</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="90">
@@ -3920,30 +3920,30 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>POLAND 1</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>AC Horsens</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>18.5</v>
+        <v>17</v>
       </c>
       <c r="G90" t="n">
-        <v>11.43</v>
+        <v>12.5</v>
       </c>
       <c r="H90" t="n">
         <v>200</v>
       </c>
       <c r="I90" t="n">
-        <v>10.86</v>
+        <v>11.88</v>
       </c>
     </row>
     <row r="91">
@@ -3959,30 +3959,30 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>ENGLAND 1</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Bandirmaspor</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Keciorengucu</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G91" t="n">
-        <v>11.76</v>
+        <v>12.5</v>
       </c>
       <c r="H91" t="n">
         <v>200</v>
       </c>
       <c r="I91" t="n">
-        <v>11.17</v>
+        <v>11.88</v>
       </c>
     </row>
     <row r="92">
@@ -3998,30 +3998,30 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>FINLAND 1</t>
+          <t>PORTUGAL 2</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Penafiel</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>FC Inter Turku</t>
+          <t>Sporting Lisbon B</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G92" t="n">
-        <v>11.11</v>
+        <v>10.53</v>
       </c>
       <c r="H92" t="n">
         <v>200</v>
       </c>
       <c r="I92" t="n">
-        <v>10.55</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93">
@@ -4037,30 +4037,30 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>VENEZUELA 1</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Hajer Club</t>
+          <t>Monagas</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Jeddah Club</t>
+          <t>Portuguesa FC</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G93" t="n">
-        <v>11.76</v>
+        <v>11.11</v>
       </c>
       <c r="H93" t="n">
         <v>200</v>
       </c>
       <c r="I93" t="n">
-        <v>11.17</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="94">
@@ -4076,17 +4076,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>DENMARK 1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Pro Vercelli</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Desenzano Calvina</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -4115,30 +4115,30 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Eyupspor</t>
+          <t>Bandirmaspor</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Gaziantep FK</t>
+          <t>Keciorengucu</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>16.5</v>
+        <v>18</v>
       </c>
       <c r="G95" t="n">
-        <v>12.9</v>
+        <v>11.76</v>
       </c>
       <c r="H95" t="n">
         <v>200</v>
       </c>
       <c r="I95" t="n">
-        <v>12.25</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="96">
@@ -4154,30 +4154,30 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>FINLAND 1</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>FC Inter Turku</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="G96" t="n">
-        <v>10.81</v>
+        <v>11.11</v>
       </c>
       <c r="H96" t="n">
         <v>200</v>
       </c>
       <c r="I96" t="n">
-        <v>10.27</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="97">
@@ -4193,30 +4193,30 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PERU 1</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Sport Boys (Per)</t>
+          <t>Hajer Club</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Cienciano</t>
+          <t>Jeddah Club</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="G97" t="n">
-        <v>11.43</v>
+        <v>11.76</v>
       </c>
       <c r="H97" t="n">
         <v>200</v>
       </c>
       <c r="I97" t="n">
-        <v>10.86</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="98">
@@ -4232,30 +4232,30 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>URUGUAY 1</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Torque</t>
+          <t>Pro Vercelli</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Wanderers (Uru)</t>
+          <t>Desenzano Calvina</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
       <c r="G98" t="n">
-        <v>10.81</v>
+        <v>11.43</v>
       </c>
       <c r="H98" t="n">
         <v>200</v>
       </c>
       <c r="I98" t="n">
-        <v>10.27</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="99">
@@ -4271,30 +4271,30 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>TURKEY 1</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Sariyer G.K.</t>
+          <t>Eyupspor</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Batman Petrolspor</t>
+          <t>Gaziantep FK</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>19</v>
+        <v>16.5</v>
       </c>
       <c r="G99" t="n">
-        <v>11.11</v>
+        <v>12.9</v>
       </c>
       <c r="H99" t="n">
         <v>200</v>
       </c>
       <c r="I99" t="n">
-        <v>10.55</v>
+        <v>12.25</v>
       </c>
     </row>
     <row r="100">
@@ -4310,30 +4310,30 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>ITALY 1</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Van Buyuksehir Belediyespor</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Istanbulspor</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="G100" t="n">
-        <v>11.11</v>
+        <v>10.81</v>
       </c>
       <c r="H100" t="n">
         <v>200</v>
       </c>
       <c r="I100" t="n">
-        <v>10.55</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="101">
@@ -4349,17 +4349,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>PERU 1</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>EC Vitoria Salvador</t>
+          <t>Sport Boys (Per)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Cienciano</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -4388,30 +4388,30 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>URUGUAY 1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Torque</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Nautico PE</t>
+          <t>Wanderers (Uru)</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="G102" t="n">
-        <v>11.76</v>
+        <v>10.81</v>
       </c>
       <c r="H102" t="n">
         <v>200</v>
       </c>
       <c r="I102" t="n">
-        <v>11.17</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="103">
@@ -4427,30 +4427,30 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ITALY 2</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Cesena</t>
+          <t>Sariyer G.K.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>Batman Petrolspor</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G103" t="n">
-        <v>11.76</v>
+        <v>11.11</v>
       </c>
       <c r="H103" t="n">
         <v>200</v>
       </c>
       <c r="I103" t="n">
-        <v>11.17</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="104">
@@ -4466,30 +4466,30 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Grosseto</t>
+          <t>Van Buyuksehir Belediyespor</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Spezia</t>
+          <t>Istanbulspor</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G104" t="n">
-        <v>11.76</v>
+        <v>11.11</v>
       </c>
       <c r="H104" t="n">
         <v>200</v>
       </c>
       <c r="I104" t="n">
-        <v>11.17</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="105">
@@ -4505,30 +4505,30 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>PARAGUAY 1</t>
+          <t>BRAZIL 1</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Olimpia</t>
+          <t>EC Vitoria Salvador</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Cerro Porteno</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>20</v>
+        <v>18.5</v>
       </c>
       <c r="G105" t="n">
-        <v>10.53</v>
+        <v>11.43</v>
       </c>
       <c r="H105" t="n">
         <v>200</v>
       </c>
       <c r="I105" t="n">
-        <v>10</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="106">
@@ -4544,30 +4544,30 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Nautico PE</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="G106" t="n">
-        <v>12.12</v>
+        <v>11.76</v>
       </c>
       <c r="H106" t="n">
         <v>200</v>
       </c>
       <c r="I106" t="n">
-        <v>11.51</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="107">
@@ -4583,30 +4583,30 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cesena</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Sampdoria</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G107" t="n">
-        <v>10.53</v>
+        <v>11.76</v>
       </c>
       <c r="H107" t="n">
         <v>200</v>
       </c>
       <c r="I107" t="n">
-        <v>10</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="108">
@@ -4622,30 +4622,30 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>ITALY 3</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Grosseto</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Spezia</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G108" t="n">
-        <v>11.11</v>
+        <v>11.76</v>
       </c>
       <c r="H108" t="n">
         <v>200</v>
       </c>
       <c r="I108" t="n">
-        <v>10.55</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="109">
@@ -4661,29 +4661,185 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
+          <t>PARAGUAY 1</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Olimpia</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Cerro Porteno</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>20</v>
+      </c>
+      <c r="G109" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="H109" t="n">
+        <v>200</v>
+      </c>
+      <c r="I109" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SPAIN 2</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G110" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="H110" t="n">
+        <v>200</v>
+      </c>
+      <c r="I110" t="n">
+        <v>11.51</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>20</v>
+      </c>
+      <c r="G111" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="H111" t="n">
+        <v>200</v>
+      </c>
+      <c r="I111" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BRAZIL 1</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>19</v>
+      </c>
+      <c r="G112" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="H112" t="n">
+        <v>200</v>
+      </c>
+      <c r="I112" t="n">
+        <v>10.55</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
           <t>COLOMBIA 1</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>Junior FC Barranquilla</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>Once Caldas</t>
         </is>
       </c>
-      <c r="F109" t="n">
+      <c r="F113" t="n">
         <v>18.5</v>
       </c>
-      <c r="G109" t="n">
+      <c r="G113" t="n">
         <v>11.43</v>
       </c>
-      <c r="H109" t="n">
-        <v>200</v>
-      </c>
-      <c r="I109" t="n">
+      <c r="H113" t="n">
+        <v>200</v>
+      </c>
+      <c r="I113" t="n">
         <v>10.86</v>
       </c>
     </row>

</xml_diff>